<commit_message>
GRUPO de ID por solicitação
</commit_message>
<xml_diff>
--- a/templates/ModeloSolicitacaoMob.xlsx
+++ b/templates/ModeloSolicitacaoMob.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vestas-my.sharepoint.com/personal/sapsd_vestas_com/Documents/Documents/GIT/SolicitadorMobilizacao-BR4/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vestas-my.sharepoint.com/personal/sapsd_vestas_com/Documents/Documents/GIT/SolicitadorMobilizacao/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="624" documentId="13_ncr:1_{FA8B678E-4D54-44A7-89A1-E9B1243370E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FCCDBC0-0A86-408E-9EB7-BAF815DD15C3}"/>
+  <xr:revisionPtr revIDLastSave="205" documentId="13_ncr:1_{497A9393-BE6E-47F5-975F-D8108371F6DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B2F7DF6-F91D-4E7B-99D1-002C3A5BFF5F}"/>
   <bookViews>
-    <workbookView xWindow="-11850" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11850" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PESSOAS" sheetId="1" r:id="rId1"/>
     <sheet name="EQUIPAMENTOS" sheetId="2" r:id="rId2"/>
-    <sheet name="LEGENDA" sheetId="4" r:id="rId3"/>
+    <sheet name="LEGENDA" sheetId="4" state="hidden" r:id="rId3"/>
     <sheet name="LISTA SUSPENSA" sheetId="3" state="hidden" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="271">
   <si>
     <t>SOLICITANTEINICIAIS</t>
   </si>
@@ -837,6 +837,15 @@
   </si>
   <si>
     <t>Equip. Placa / Num. Série [Equip_x005F_x002e_Placa_x005F_x002f_Num_x002]</t>
+  </si>
+  <si>
+    <t>GRUPO</t>
+  </si>
+  <si>
+    <t>SENAI</t>
+  </si>
+  <si>
+    <t>SIMM Soluções</t>
   </si>
   <si>
     <t>Tomé</t>
@@ -994,7 +1003,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -1021,17 +1030,27 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="18">
     <dxf>
       <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1187,6 +1206,10 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -1207,35 +1230,45 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A960259-2F5D-4C27-91C2-AFF5E9FD9747}" name="Table1" displayName="Table1" ref="A1:M50" totalsRowShown="0" dataDxfId="15">
-  <autoFilter ref="A1:M50" xr:uid="{4A960259-2F5D-4C27-91C2-AFF5E9FD9747}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{4826DB81-466A-4500-9D0B-E285A1D12845}" name="Solicitante [SOLICITANTEINICIAIS]" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{39336303-107B-40A8-B569-6106ACA06F79}" name="Parque Destino [Parque]" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{240B30AE-1961-4D52-95E4-2068626BF8D6}" name="Data Acesso [DATADOACESSO]" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{AB894E94-7977-4290-B724-C76AED6A9E2C}" name="Data Desmobilização [DataDesmobiliza_x005f_x00e7__x005f_x00e3_o]" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{B843020A-A81E-4644-9E5B-7B3F6AC4777B}" name="Fornecedor [FORNECEDOR]" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{505BDD86-8C85-445C-ADA4-21D872FE4F1E}" name="Tipo Mobilização [TipoMobiliza_x005f_x00e7__x005f_x00e3_o]" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{02D4BDF3-E850-4441-8164-5FE6780A4B6D}" name="Tipo de Atividade [TIPODEATIVIDADE]" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{52B836D7-BB07-4119-8E33-A64A0D765638}" name="Especificação técnica/Experiência [Especifica_x005f_x00e7__x005f_x00e3_ot_x00e9]" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{C4BD4A19-77B0-47C6-87BB-7C7B2896D696}" name="Necessário Carro? [Necess_x005f_x00e1_rioCarro_x005f_x003f_]" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{811A5AF1-B1B7-4467-ACC1-B080F1093DE0}" name="Tipo de Carro [TipodeCarro]" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{A2694C6F-6F39-4134-93E9-81D4E1032ED9}" name="Detalhamento da Atividade [DETALHAMENTODAATIVIDADE]" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{5D43A1D2-B98A-430D-A764-4891FF049847}" name="Função [FUN_x005f_x00c7__x005f_x00c3_O]" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{82088B2D-F67B-492D-974F-EB28FCE24D7A}" name="Colaborador [COLABORADOR_]" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A960259-2F5D-4C27-91C2-AFF5E9FD9747}" name="Table1" displayName="Table1" ref="A1:N47" totalsRowShown="0" dataDxfId="17">
+  <autoFilter ref="A1:N47" xr:uid="{4A960259-2F5D-4C27-91C2-AFF5E9FD9747}"/>
+  <tableColumns count="14">
+    <tableColumn id="15" xr3:uid="{B0122549-AEFC-47C0-B9D2-3D3B0B9A316F}" name="GRUPO" dataDxfId="16"/>
+    <tableColumn id="14" xr3:uid="{0AF23745-21D0-410B-A887-D2086E1BC51B}" name="Solicitante [SOLICITANTEINICIAIS]" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{39336303-107B-40A8-B569-6106ACA06F79}" name="Parque Destino [Parque]" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{240B30AE-1961-4D52-95E4-2068626BF8D6}" name="Data Acesso [DATADOACESSO]" dataDxfId="13">
+      <calculatedColumnFormula>TODAY()</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{AB894E94-7977-4290-B724-C76AED6A9E2C}" name="Data Desmobilização [DataDesmobiliza_x005f_x00e7__x005f_x00e3_o]" dataDxfId="12">
+      <calculatedColumnFormula>TODAY()+25</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{B843020A-A81E-4644-9E5B-7B3F6AC4777B}" name="Fornecedor [FORNECEDOR]" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{505BDD86-8C85-445C-ADA4-21D872FE4F1E}" name="Tipo Mobilização [TipoMobiliza_x005f_x00e7__x005f_x00e3_o]" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{02D4BDF3-E850-4441-8164-5FE6780A4B6D}" name="Tipo de Atividade [TIPODEATIVIDADE]" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{52B836D7-BB07-4119-8E33-A64A0D765638}" name="Especificação técnica/Experiência [Especifica_x005f_x00e7__x005f_x00e3_ot_x00e9]" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{C4BD4A19-77B0-47C6-87BB-7C7B2896D696}" name="Necessário Carro? [Necess_x005f_x00e1_rioCarro_x005f_x003f_]" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{811A5AF1-B1B7-4467-ACC1-B080F1093DE0}" name="Tipo de Carro [TipodeCarro]" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{A2694C6F-6F39-4134-93E9-81D4E1032ED9}" name="Detalhamento da Atividade [DETALHAMENTODAATIVIDADE]" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{5D43A1D2-B98A-430D-A764-4891FF049847}" name="Função [FUN_x005f_x00c7__x005f_x00c3_O]" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{82088B2D-F67B-492D-974F-EB28FCE24D7A}" name="Colaborador [COLABORADOR_]" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E8379FD7-EC41-4E83-95E0-6B6CE0A80AD0}" name="Table3" displayName="Table3" ref="A1:I50" totalsRowShown="0">
-  <autoFilter ref="A1:I50" xr:uid="{E8379FD7-EC41-4E83-95E0-6B6CE0A80AD0}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{861EC4AE-4118-4245-AB5D-EAFC76888E80}" name="Solicitante [SOLICITANTEINICIAIS]"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E8379FD7-EC41-4E83-95E0-6B6CE0A80AD0}" name="Table3" displayName="Table3" ref="A1:J47" totalsRowShown="0">
+  <autoFilter ref="A1:J47" xr:uid="{E8379FD7-EC41-4E83-95E0-6B6CE0A80AD0}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{861EC4AE-4118-4245-AB5D-EAFC76888E80}" name="GRUPO" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{01A22A7C-F406-49B6-9CCE-3865E85F7239}" name="Solicitante [SOLICITANTEINICIAIS]"/>
     <tableColumn id="2" xr3:uid="{84B8AD55-9A13-4BA3-8F43-848B16639D31}" name="Parque Destino [Parque]"/>
-    <tableColumn id="3" xr3:uid="{4F6814DD-4460-428D-B511-32E248131F6E}" name="Data Acesso [DATADOACESSO]" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{83E74907-E643-4102-B744-9C1475EDD631}" name="Data Desmobilização [DataDesmobiliza_x005f_x00e7__x005f_x00e3_o]" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{4F6814DD-4460-428D-B511-32E248131F6E}" name="Data Acesso [DATADOACESSO]" dataDxfId="1">
+      <calculatedColumnFormula>TODAY()</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{83E74907-E643-4102-B744-9C1475EDD631}" name="Data Desmobilização [DataDesmobiliza_x005f_x00e7__x005f_x00e3_o]" dataDxfId="0">
+      <calculatedColumnFormula>TODAY()+20</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="4" xr3:uid="{771729CF-CE59-4856-B391-1616C73F75F1}" name="Fornecedor [FORNECEDOR]"/>
     <tableColumn id="5" xr3:uid="{CC7230EF-82B8-4B4C-95FC-B7BA91D7FEF5}" name="Tipo Mobilização [TipoMobiliza_x005f_x00e7__x005f_x00e3_o]"/>
     <tableColumn id="6" xr3:uid="{50A55B65-C50D-40DA-8867-1D55BB2EF9C8}" name="Equipamento [Equipamento]"/>
@@ -1563,863 +1596,876 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="32.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="52.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="33.54296875" customWidth="1"/>
-    <col min="11" max="11" width="29.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="21.6328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="40.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.08984375" style="16" customWidth="1"/>
+    <col min="2" max="2" width="32.26953125" customWidth="1"/>
+    <col min="3" max="3" width="24.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="33.54296875" customWidth="1"/>
+    <col min="12" max="12" width="29.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="40.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A1" s="16" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1" t="s">
         <v>251</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>252</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>253</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>254</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>255</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>256</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>257</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>258</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>259</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>260</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>261</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>262</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="4"/>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" s="17"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="3"/>
       <c r="D2" s="4"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="5"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="3"/>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
-      <c r="M2" s="3"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="4"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="3"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" s="17"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="3"/>
       <c r="D3" s="4"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="5"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="3"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
-      <c r="M3" s="3"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="4"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="3"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" s="17"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="3"/>
       <c r="D4" s="4"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="5"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="3"/>
       <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
       <c r="L4" s="5"/>
-      <c r="M4" s="3"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="4"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="3"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" s="17"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="3"/>
       <c r="D5" s="4"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="5"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="3"/>
       <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="3"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="4"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="3"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6" s="17"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="3"/>
       <c r="D6" s="4"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="5"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="3"/>
       <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="3"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7" s="2"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="4"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="3"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" s="17"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="3"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="5"/>
-      <c r="I7" s="5"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="5"/>
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
-      <c r="M7" s="3"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8" s="2"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="4"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="3"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" s="17"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="3"/>
       <c r="D8" s="4"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="5"/>
-      <c r="I8" s="5"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="5"/>
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
       <c r="L8" s="5"/>
-      <c r="M8" s="3"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="4"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="3"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" s="17"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="3"/>
       <c r="D9" s="4"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="5"/>
-      <c r="I9" s="5"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="5"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
       <c r="L9" s="5"/>
-      <c r="M9" s="3"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="4"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="3"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" s="17"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="3"/>
       <c r="D10" s="4"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="5"/>
-      <c r="I10" s="5"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
-      <c r="M10" s="3"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="4"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="3"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" s="17"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="3"/>
       <c r="D11" s="4"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="5"/>
-      <c r="I11" s="5"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
-      <c r="M11" s="3"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A12" s="2"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="4"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="3"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12" s="17"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="3"/>
       <c r="D12" s="4"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="5"/>
-      <c r="I12" s="5"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="5"/>
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
-      <c r="M12" s="3"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A13" s="2"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="4"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="3"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" s="17"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="3"/>
       <c r="D13" s="4"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="5"/>
-      <c r="I13" s="5"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="5"/>
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
-      <c r="M13" s="3"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14" s="2"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="3"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A14" s="18"/>
       <c r="B14" s="3"/>
-      <c r="C14" s="4"/>
+      <c r="C14" s="3"/>
       <c r="D14" s="4"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="5"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
-      <c r="M14" s="3"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A15" s="2"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="3"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A15" s="18"/>
       <c r="B15" s="3"/>
-      <c r="C15" s="4"/>
+      <c r="C15" s="3"/>
       <c r="D15" s="4"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="5"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
-      <c r="M15" s="3"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A16" s="2"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="3"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A16" s="18"/>
       <c r="B16" s="3"/>
-      <c r="C16" s="4"/>
+      <c r="C16" s="3"/>
       <c r="D16" s="4"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="5"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="5"/>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="3"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A17" s="3"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="3"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A17" s="18"/>
       <c r="B17" s="3"/>
-      <c r="C17" s="4"/>
+      <c r="C17" s="3"/>
       <c r="D17" s="4"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="5"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="3"/>
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
-      <c r="M17" s="3"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A18" s="3"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="3"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A18" s="18"/>
       <c r="B18" s="3"/>
-      <c r="C18" s="4"/>
+      <c r="C18" s="3"/>
       <c r="D18" s="4"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="5"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="3"/>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
-      <c r="M18" s="3"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A19" s="3"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="3"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A19" s="18"/>
       <c r="B19" s="3"/>
-      <c r="C19" s="4"/>
+      <c r="C19" s="3"/>
       <c r="D19" s="4"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="5"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="3"/>
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
-      <c r="M19" s="3"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A20" s="3"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="3"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A20" s="18"/>
       <c r="B20" s="3"/>
-      <c r="C20" s="4"/>
+      <c r="C20" s="3"/>
       <c r="D20" s="4"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="5"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="3"/>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
-      <c r="M20" s="3"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A21" s="3"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="3"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A21" s="18"/>
       <c r="B21" s="3"/>
-      <c r="C21" s="4"/>
+      <c r="C21" s="3"/>
       <c r="D21" s="4"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="5"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="3"/>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
-      <c r="M21" s="3"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A22" s="3"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="3"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A22" s="18"/>
       <c r="B22" s="3"/>
-      <c r="C22" s="4"/>
+      <c r="C22" s="3"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="5"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="3"/>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
-      <c r="M22" s="3"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A23" s="3"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="3"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A23" s="18"/>
       <c r="B23" s="3"/>
-      <c r="C23" s="4"/>
+      <c r="C23" s="3"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="5"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="3"/>
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
-      <c r="M23" s="3"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A24" s="3"/>
+      <c r="M23" s="5"/>
+      <c r="N23" s="3"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A24" s="18"/>
       <c r="B24" s="3"/>
-      <c r="C24" s="4"/>
+      <c r="C24" s="3"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="5"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="3"/>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
-      <c r="M24" s="3"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A25" s="3"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="3"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A25" s="18"/>
       <c r="B25" s="3"/>
-      <c r="C25" s="4"/>
+      <c r="C25" s="3"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="5"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="3"/>
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
-      <c r="M25" s="3"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A26" s="3"/>
+      <c r="M25" s="5"/>
+      <c r="N25" s="3"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A26" s="18"/>
       <c r="B26" s="3"/>
-      <c r="C26" s="4"/>
+      <c r="C26" s="3"/>
       <c r="D26" s="4"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="5"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="3"/>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
-      <c r="M26" s="3"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A27" s="3"/>
+      <c r="M26" s="5"/>
+      <c r="N26" s="3"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A27" s="18"/>
       <c r="B27" s="3"/>
-      <c r="C27" s="4"/>
+      <c r="C27" s="3"/>
       <c r="D27" s="4"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="5"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="3"/>
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
       <c r="K27" s="5"/>
       <c r="L27" s="5"/>
-      <c r="M27" s="3"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A28" s="3"/>
+      <c r="M27" s="5"/>
+      <c r="N27" s="3"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A28" s="18"/>
       <c r="B28" s="3"/>
-      <c r="C28" s="4"/>
+      <c r="C28" s="3"/>
       <c r="D28" s="4"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="5"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="3"/>
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5"/>
       <c r="L28" s="5"/>
-      <c r="M28" s="3"/>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A29" s="3"/>
+      <c r="M28" s="5"/>
+      <c r="N28" s="3"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A29" s="18"/>
       <c r="B29" s="3"/>
-      <c r="C29" s="4"/>
+      <c r="C29" s="3"/>
       <c r="D29" s="4"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="5"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="3"/>
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
       <c r="K29" s="5"/>
       <c r="L29" s="5"/>
-      <c r="M29" s="3"/>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A30" s="3"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="3"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A30" s="18"/>
       <c r="B30" s="3"/>
-      <c r="C30" s="4"/>
+      <c r="C30" s="3"/>
       <c r="D30" s="4"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="5"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="3"/>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5"/>
       <c r="L30" s="5"/>
-      <c r="M30" s="3"/>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A31" s="3"/>
+      <c r="M30" s="5"/>
+      <c r="N30" s="3"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A31" s="18"/>
       <c r="B31" s="3"/>
-      <c r="C31" s="4"/>
+      <c r="C31" s="3"/>
       <c r="D31" s="4"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="5"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="3"/>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
       <c r="K31" s="5"/>
       <c r="L31" s="5"/>
-      <c r="M31" s="3"/>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A32" s="3"/>
+      <c r="M31" s="5"/>
+      <c r="N31" s="3"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A32" s="18"/>
       <c r="B32" s="3"/>
-      <c r="C32" s="4"/>
+      <c r="C32" s="3"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="5"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="3"/>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
       <c r="K32" s="5"/>
       <c r="L32" s="5"/>
-      <c r="M32" s="3"/>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A33" s="3"/>
+      <c r="M32" s="5"/>
+      <c r="N32" s="3"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A33" s="18"/>
       <c r="B33" s="3"/>
-      <c r="C33" s="4"/>
+      <c r="C33" s="3"/>
       <c r="D33" s="4"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="5"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="3"/>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
       <c r="K33" s="5"/>
       <c r="L33" s="5"/>
-      <c r="M33" s="3"/>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A34" s="3"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="3"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A34" s="18"/>
       <c r="B34" s="3"/>
-      <c r="C34" s="4"/>
+      <c r="C34" s="3"/>
       <c r="D34" s="4"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="5"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="3"/>
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
       <c r="K34" s="5"/>
       <c r="L34" s="5"/>
-      <c r="M34" s="3"/>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A35" s="3"/>
+      <c r="M34" s="5"/>
+      <c r="N34" s="3"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A35" s="18"/>
       <c r="B35" s="3"/>
-      <c r="C35" s="4"/>
+      <c r="C35" s="3"/>
       <c r="D35" s="4"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="5"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="3"/>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
       <c r="K35" s="5"/>
       <c r="L35" s="5"/>
-      <c r="M35" s="3"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A36" s="3"/>
+      <c r="M35" s="5"/>
+      <c r="N35" s="3"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A36" s="18"/>
       <c r="B36" s="3"/>
-      <c r="C36" s="4"/>
+      <c r="C36" s="3"/>
       <c r="D36" s="4"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="5"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="3"/>
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
       <c r="K36" s="5"/>
       <c r="L36" s="5"/>
-      <c r="M36" s="3"/>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A37" s="3"/>
+      <c r="M36" s="5"/>
+      <c r="N36" s="3"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A37" s="18"/>
       <c r="B37" s="3"/>
-      <c r="C37" s="4"/>
+      <c r="C37" s="3"/>
       <c r="D37" s="4"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="5"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="3"/>
       <c r="H37" s="5"/>
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
       <c r="K37" s="5"/>
       <c r="L37" s="5"/>
-      <c r="M37" s="3"/>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A38" s="3"/>
+      <c r="M37" s="5"/>
+      <c r="N37" s="3"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A38" s="18"/>
       <c r="B38" s="3"/>
-      <c r="C38" s="4"/>
+      <c r="C38" s="3"/>
       <c r="D38" s="4"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="3"/>
-      <c r="G38" s="5"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="3"/>
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
       <c r="K38" s="5"/>
       <c r="L38" s="5"/>
-      <c r="M38" s="3"/>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A39" s="3"/>
+      <c r="M38" s="5"/>
+      <c r="N38" s="3"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A39" s="18"/>
       <c r="B39" s="3"/>
-      <c r="C39" s="4"/>
+      <c r="C39" s="3"/>
       <c r="D39" s="4"/>
-      <c r="E39" s="5"/>
-      <c r="F39" s="3"/>
-      <c r="G39" s="5"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="3"/>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
       <c r="K39" s="5"/>
       <c r="L39" s="5"/>
-      <c r="M39" s="3"/>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A40" s="3"/>
+      <c r="M39" s="5"/>
+      <c r="N39" s="3"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A40" s="18"/>
       <c r="B40" s="3"/>
-      <c r="C40" s="4"/>
+      <c r="C40" s="3"/>
       <c r="D40" s="4"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="3"/>
-      <c r="G40" s="5"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="3"/>
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
       <c r="K40" s="5"/>
       <c r="L40" s="5"/>
-      <c r="M40" s="3"/>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A41" s="3"/>
+      <c r="M40" s="5"/>
+      <c r="N40" s="3"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A41" s="18"/>
       <c r="B41" s="3"/>
-      <c r="C41" s="4"/>
+      <c r="C41" s="3"/>
       <c r="D41" s="4"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="3"/>
-      <c r="G41" s="5"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="3"/>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
       <c r="K41" s="5"/>
       <c r="L41" s="5"/>
-      <c r="M41" s="3"/>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A42" s="3"/>
+      <c r="M41" s="5"/>
+      <c r="N41" s="3"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A42" s="18"/>
       <c r="B42" s="3"/>
-      <c r="C42" s="4"/>
+      <c r="C42" s="3"/>
       <c r="D42" s="4"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="3"/>
-      <c r="G42" s="5"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="3"/>
       <c r="H42" s="5"/>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
       <c r="K42" s="5"/>
       <c r="L42" s="5"/>
-      <c r="M42" s="3"/>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A43" s="3"/>
+      <c r="M42" s="5"/>
+      <c r="N42" s="3"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A43" s="18"/>
       <c r="B43" s="3"/>
-      <c r="C43" s="4"/>
+      <c r="C43" s="3"/>
       <c r="D43" s="4"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="3"/>
-      <c r="G43" s="5"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="3"/>
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
       <c r="K43" s="5"/>
       <c r="L43" s="5"/>
-      <c r="M43" s="3"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A44" s="3"/>
+      <c r="M43" s="5"/>
+      <c r="N43" s="3"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A44" s="18"/>
       <c r="B44" s="3"/>
-      <c r="C44" s="4"/>
+      <c r="C44" s="3"/>
       <c r="D44" s="4"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="3"/>
-      <c r="G44" s="5"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="3"/>
       <c r="H44" s="5"/>
       <c r="I44" s="5"/>
       <c r="J44" s="5"/>
       <c r="K44" s="5"/>
       <c r="L44" s="5"/>
-      <c r="M44" s="3"/>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A45" s="3"/>
+      <c r="M44" s="5"/>
+      <c r="N44" s="3"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A45" s="18"/>
       <c r="B45" s="3"/>
-      <c r="C45" s="4"/>
+      <c r="C45" s="3"/>
       <c r="D45" s="4"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="3"/>
-      <c r="G45" s="5"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="3"/>
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
       <c r="K45" s="5"/>
       <c r="L45" s="5"/>
-      <c r="M45" s="3"/>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A46" s="3"/>
+      <c r="M45" s="5"/>
+      <c r="N45" s="3"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A46" s="18"/>
       <c r="B46" s="3"/>
-      <c r="C46" s="4"/>
+      <c r="C46" s="3"/>
       <c r="D46" s="4"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="5"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="3"/>
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
       <c r="K46" s="5"/>
       <c r="L46" s="5"/>
-      <c r="M46" s="3"/>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A47" s="3"/>
+      <c r="M46" s="5"/>
+      <c r="N46" s="3"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A47" s="18"/>
       <c r="B47" s="3"/>
-      <c r="C47" s="4"/>
+      <c r="C47" s="3"/>
       <c r="D47" s="4"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="5"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="3"/>
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
       <c r="K47" s="5"/>
       <c r="L47" s="5"/>
-      <c r="M47" s="3"/>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A48" s="3"/>
+      <c r="M47" s="5"/>
+      <c r="N47" s="3"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A48" s="18"/>
       <c r="B48" s="3"/>
-      <c r="C48" s="4"/>
+      <c r="C48" s="3"/>
       <c r="D48" s="4"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="5"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="3"/>
       <c r="H48" s="5"/>
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
       <c r="K48" s="5"/>
       <c r="L48" s="5"/>
-      <c r="M48" s="3"/>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A49" s="3"/>
+      <c r="M48" s="5"/>
+      <c r="N48" s="3"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A49" s="18"/>
       <c r="B49" s="3"/>
-      <c r="C49" s="4"/>
+      <c r="C49" s="3"/>
       <c r="D49" s="4"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="3"/>
-      <c r="G49" s="5"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="3"/>
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
       <c r="K49" s="5"/>
       <c r="L49" s="5"/>
-      <c r="M49" s="3"/>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A50" s="3"/>
+      <c r="M49" s="5"/>
+      <c r="N49" s="3"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A50" s="18"/>
       <c r="B50" s="3"/>
-      <c r="C50" s="4"/>
+      <c r="C50" s="3"/>
       <c r="D50" s="4"/>
-      <c r="E50" s="5"/>
-      <c r="F50" s="3"/>
-      <c r="G50" s="5"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="3"/>
       <c r="H50" s="5"/>
       <c r="I50" s="5"/>
       <c r="J50" s="5"/>
       <c r="K50" s="5"/>
       <c r="L50" s="5"/>
-      <c r="M50" s="3"/>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A51" s="3"/>
+      <c r="M50" s="5"/>
+      <c r="N50" s="3"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A51" s="18"/>
       <c r="B51" s="3"/>
-      <c r="C51" s="4"/>
+      <c r="C51" s="3"/>
       <c r="D51" s="4"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="3"/>
-      <c r="G51" s="5"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="3"/>
       <c r="H51" s="5"/>
       <c r="I51" s="5"/>
       <c r="J51" s="5"/>
       <c r="K51" s="5"/>
       <c r="L51" s="5"/>
-      <c r="M51" s="3"/>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4"/>
-      <c r="E52" s="5"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="5"/>
-      <c r="H52" s="5"/>
-      <c r="I52" s="5"/>
-      <c r="J52" s="5"/>
-      <c r="K52" s="5"/>
-      <c r="L52" s="5"/>
-      <c r="M52" s="3"/>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="4"/>
-      <c r="E53" s="5"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="5"/>
-      <c r="H53" s="5"/>
-      <c r="I53" s="5"/>
-      <c r="J53" s="5"/>
-      <c r="K53" s="5"/>
-      <c r="L53" s="5"/>
-      <c r="M53" s="3"/>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="5"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="5"/>
-      <c r="H54" s="5"/>
-      <c r="I54" s="5"/>
-      <c r="J54" s="5"/>
-      <c r="K54" s="5"/>
-      <c r="L54" s="5"/>
-      <c r="M54" s="3"/>
+      <c r="M51" s="5"/>
+      <c r="N51" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:D50" xr:uid="{4DA6711F-7DE6-41AC-88D1-6B374A17C2EF}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:E47" xr:uid="{4DA6711F-7DE6-41AC-88D1-6B374A17C2EF}">
       <formula1>46023</formula1>
       <formula2>73415</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Classification: Confidential</oddFooter>
   </headerFooter>
+  <ignoredErrors>
+    <ignoredError sqref="D2:E47" calculatedColumn="1"/>
+  </ignoredErrors>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2428,73 +2474,73 @@
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$A$2:$A$54</xm:f>
           </x14:formula1>
-          <xm:sqref>B7:B1048576</xm:sqref>
+          <xm:sqref>C4:C1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{792BB204-51C2-4508-91DA-F0ADAB177D39}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$B$2:$B$100</xm:f>
           </x14:formula1>
-          <xm:sqref>E7:E1048576</xm:sqref>
+          <xm:sqref>F4:F1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A67059F1-3AFA-4842-8E84-ED670BFB9B1B}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$D$2:$D$10</xm:f>
           </x14:formula1>
-          <xm:sqref>G49:H1048576 G7:G48</xm:sqref>
+          <xm:sqref>H46:I1048576 H4:H45</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{516B2B10-5C85-420F-A84E-F75CBB23B990}">
+          <x14:formula1>
+            <xm:f>'LISTA SUSPENSA'!$C$2:$C$120</xm:f>
+          </x14:formula1>
+          <xm:sqref>M4:M1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{CB39C5A8-B3BF-463B-8FBA-30C423AE4D8E}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$E$2:$E$3</xm:f>
           </x14:formula1>
-          <xm:sqref>I2:I50</xm:sqref>
+          <xm:sqref>J2:J47</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2C7BD5C7-09B1-4161-BAEB-8AE58FB21DFA}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$G$2:$G$3</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F50</xm:sqref>
+          <xm:sqref>G2:G47</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F4EE3F9A-A30D-424E-B756-362F17268AF4}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$F$2:$F$4</xm:f>
           </x14:formula1>
-          <xm:sqref>J2:J50</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{516B2B10-5C85-420F-A84E-F75CBB23B990}">
-          <x14:formula1>
-            <xm:f>'LISTA SUSPENSA'!$C$2:$C$120</xm:f>
-          </x14:formula1>
-          <xm:sqref>L7:L1048576</xm:sqref>
+          <xm:sqref>K2:K47</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{24746D03-D41F-45BC-A65E-F2441DACE54C}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$C$2:$C$100</xm:f>
           </x14:formula1>
-          <xm:sqref>L2:L50</xm:sqref>
+          <xm:sqref>M2:M47</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6A30AE29-97EB-4E69-B196-8C58355F1F0D}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$A$2:$A$500</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B6</xm:sqref>
+          <xm:sqref>C2:C3</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3E5A2525-B7D0-4670-9577-5A78863D2E4E}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$B$2:$B$500</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E6</xm:sqref>
+          <xm:sqref>F2:F3</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{670867F6-90AF-4EDD-901F-C6B148C42EC2}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$D$2:$D$100</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G6</xm:sqref>
+          <xm:sqref>H2:H3</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E7608E0F-4567-4C9F-AD49-98F5DDBCABE2}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$C$2:$C$500</xm:f>
           </x14:formula1>
-          <xm:sqref>L2:L6</xm:sqref>
+          <xm:sqref>M2:M3</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2504,280 +2550,263 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.453125" customWidth="1"/>
-    <col min="2" max="2" width="17.1796875" customWidth="1"/>
-    <col min="3" max="3" width="16.6328125" customWidth="1"/>
-    <col min="4" max="4" width="32.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.7265625" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="39.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="41.81640625" customWidth="1"/>
+    <col min="1" max="1" width="20.453125" style="16" customWidth="1"/>
+    <col min="2" max="2" width="32.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" customWidth="1"/>
+    <col min="4" max="4" width="16.6328125" customWidth="1"/>
+    <col min="5" max="5" width="32.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.7265625" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="39.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="41.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1" s="16" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1" t="s">
         <v>251</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>252</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>253</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>255</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>256</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>264</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>265</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C2" s="1"/>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C3" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C4" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C5" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C6" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C7" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C8" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C9" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C10" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C11" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C12" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C13" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C14" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C15" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C16" s="1"/>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C17" s="1"/>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C18" s="1"/>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C19" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C20" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D20" s="1"/>
-    </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C21" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D21" s="1"/>
-    </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C22" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D22" s="1"/>
-    </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C23" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D23" s="1"/>
-    </row>
-    <row r="24" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C24" s="1"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D24" s="1"/>
-    </row>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C25" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D25" s="1"/>
-    </row>
-    <row r="26" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C26" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D26" s="1"/>
-    </row>
-    <row r="27" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C27" s="1"/>
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D27" s="1"/>
-    </row>
-    <row r="28" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C28" s="1"/>
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D28" s="1"/>
-    </row>
-    <row r="29" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C29" s="1"/>
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D29" s="1"/>
-    </row>
-    <row r="30" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C30" s="1"/>
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D30" s="1"/>
-    </row>
-    <row r="31" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C31" s="1"/>
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D31" s="1"/>
-    </row>
-    <row r="32" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C32" s="1"/>
+      <c r="E31" s="1"/>
+    </row>
+    <row r="32" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D32" s="1"/>
-    </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C33" s="1"/>
+      <c r="E32" s="1"/>
+    </row>
+    <row r="33" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D33" s="1"/>
-    </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C34" s="1"/>
+      <c r="E33" s="1"/>
+    </row>
+    <row r="34" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D34" s="1"/>
-    </row>
-    <row r="35" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C35" s="1"/>
+      <c r="E34" s="1"/>
+    </row>
+    <row r="35" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D35" s="1"/>
-    </row>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C36" s="1"/>
+      <c r="E35" s="1"/>
+    </row>
+    <row r="36" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D36" s="1"/>
-    </row>
-    <row r="37" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C37" s="1"/>
+      <c r="E36" s="1"/>
+    </row>
+    <row r="37" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D37" s="1"/>
-    </row>
-    <row r="38" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C38" s="1"/>
+      <c r="E37" s="1"/>
+    </row>
+    <row r="38" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D38" s="1"/>
-    </row>
-    <row r="39" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C39" s="1"/>
+      <c r="E38" s="1"/>
+    </row>
+    <row r="39" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D39" s="1"/>
-    </row>
-    <row r="40" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C40" s="1"/>
+      <c r="E39" s="1"/>
+    </row>
+    <row r="40" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D40" s="1"/>
-    </row>
-    <row r="41" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C41" s="1"/>
+      <c r="E40" s="1"/>
+    </row>
+    <row r="41" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D41" s="1"/>
-    </row>
-    <row r="42" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C42" s="1"/>
+      <c r="E41" s="1"/>
+    </row>
+    <row r="42" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D42" s="1"/>
-    </row>
-    <row r="43" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C43" s="1"/>
+      <c r="E42" s="1"/>
+    </row>
+    <row r="43" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D43" s="1"/>
-    </row>
-    <row r="44" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C44" s="1"/>
+      <c r="E43" s="1"/>
+    </row>
+    <row r="44" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D44" s="1"/>
-    </row>
-    <row r="45" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C45" s="1"/>
+      <c r="E44" s="1"/>
+    </row>
+    <row r="45" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D45" s="1"/>
-    </row>
-    <row r="46" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C46" s="1"/>
+      <c r="E45" s="1"/>
+    </row>
+    <row r="46" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D46" s="1"/>
-    </row>
-    <row r="47" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C47" s="1"/>
+      <c r="E46" s="1"/>
+    </row>
+    <row r="47" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D47" s="1"/>
-    </row>
-    <row r="48" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C48" s="1"/>
+      <c r="E47" s="1"/>
+    </row>
+    <row r="48" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D48" s="1"/>
-    </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C49" s="1"/>
+      <c r="E48" s="1"/>
+    </row>
+    <row r="49" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D49" s="1"/>
-    </row>
-    <row r="50" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C50" s="1"/>
+      <c r="E49" s="1"/>
+    </row>
+    <row r="50" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D50" s="1"/>
-    </row>
-    <row r="51" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C51" s="1"/>
+      <c r="E50" s="1"/>
+    </row>
+    <row r="51" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D51" s="1"/>
-    </row>
-    <row r="52" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C52" s="1"/>
+      <c r="E51" s="1"/>
+    </row>
+    <row r="52" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D52" s="1"/>
-    </row>
-    <row r="53" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C53" s="1"/>
+      <c r="E52" s="1"/>
+    </row>
+    <row r="53" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D53" s="1"/>
-    </row>
-    <row r="54" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C54" s="1"/>
-      <c r="D54" s="1"/>
-    </row>
-    <row r="55" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C55" s="1"/>
-      <c r="D55" s="1"/>
-    </row>
-    <row r="56" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C56" s="1"/>
-      <c r="D56" s="1"/>
+      <c r="E53" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
-  <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2" xr:uid="{10C8AFF6-4D9F-4C18-8D19-BE51C4DFD3ED}">
-      <formula1>46023</formula1>
-      <formula2>73415</formula2>
-    </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{0FC3B47C-98B0-4B59-9486-5C1E83968EAF}">
-      <formula1>46023</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Classification: Confidential</oddFooter>
@@ -2792,25 +2821,25 @@
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$A$2:$A$54</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B50</xm:sqref>
+          <xm:sqref>C2:C47</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{72E0B5F8-B447-4DC3-B239-23DF70B480F7}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$B$2:$B$54</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E50</xm:sqref>
+          <xm:sqref>F2:F47</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A6666B5F-2F9F-4644-84B0-2E312873DB5C}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$G$2:$G$3</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F50</xm:sqref>
+          <xm:sqref>G2:G47</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0FF491BF-8D47-4C39-BF20-EFEAC662263A}">
           <x14:formula1>
             <xm:f>'LISTA SUSPENSA'!$H$2:$H$6</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H50</xm:sqref>
+          <xm:sqref>I2:I47</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3716,7 +3745,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B60" t="s">
-        <v>235</v>
+        <v>268</v>
       </c>
       <c r="C60" s="7" t="s">
         <v>166</v>
@@ -3724,7 +3753,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B61" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C61" s="7" t="s">
         <v>211</v>
@@ -3732,7 +3761,7 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B62" t="s">
-        <v>229</v>
+        <v>269</v>
       </c>
       <c r="C62" s="7" t="s">
         <v>212</v>
@@ -3740,7 +3769,7 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B63" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="C63" s="7" t="s">
         <v>213</v>
@@ -3748,7 +3777,7 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B64" t="s">
-        <v>54</v>
+        <v>229</v>
       </c>
       <c r="C64" s="7" t="s">
         <v>214</v>
@@ -3756,7 +3785,7 @@
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B65" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C65" s="7" t="s">
         <v>215</v>
@@ -3764,7 +3793,7 @@
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C66" s="7" t="s">
         <v>241</v>
@@ -3772,7 +3801,7 @@
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
-        <v>56</v>
+        <v>232</v>
       </c>
       <c r="C67" s="7" t="s">
         <v>242</v>
@@ -3780,7 +3809,7 @@
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C68" s="7" t="s">
         <v>243</v>
@@ -3788,7 +3817,7 @@
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C69" s="7" t="s">
         <v>244</v>
@@ -3796,7 +3825,7 @@
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
-        <v>267</v>
+        <v>57</v>
       </c>
       <c r="C70" s="7" t="s">
         <v>245</v>
@@ -3804,110 +3833,116 @@
     </row>
     <row r="71" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B71" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C71" s="7"/>
     </row>
     <row r="72" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B72" t="s">
-        <v>60</v>
+        <v>270</v>
       </c>
       <c r="C72" s="7"/>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B73" t="s">
-        <v>230</v>
+        <v>59</v>
       </c>
       <c r="C73" s="7"/>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B74" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C74" s="7"/>
     </row>
     <row r="75" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B75" t="s">
-        <v>62</v>
+        <v>230</v>
       </c>
       <c r="C75" s="7"/>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B76" t="s">
-        <v>231</v>
+        <v>61</v>
       </c>
       <c r="C76" s="7"/>
     </row>
     <row r="77" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B77" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C77" s="7"/>
     </row>
     <row r="78" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B78" t="s">
-        <v>64</v>
+        <v>231</v>
       </c>
       <c r="C78" s="7"/>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B79" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C79" s="7"/>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
+        <v>64</v>
+      </c>
+      <c r="C80" s="7"/>
+    </row>
+    <row r="81" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B81" t="s">
+        <v>65</v>
+      </c>
+      <c r="C81" s="7"/>
+    </row>
+    <row r="82" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B82" t="s">
         <v>66</v>
       </c>
-      <c r="C80" s="7"/>
-    </row>
-    <row r="81" spans="3:3" x14ac:dyDescent="0.35">
-      <c r="C81" s="7"/>
-    </row>
-    <row r="82" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C82" s="7"/>
     </row>
-    <row r="83" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C83" s="7"/>
     </row>
-    <row r="84" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C84" s="7"/>
     </row>
-    <row r="85" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C85" s="7"/>
     </row>
-    <row r="86" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C86" s="7"/>
     </row>
-    <row r="87" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C87" s="7"/>
     </row>
-    <row r="88" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C88" s="7"/>
     </row>
-    <row r="89" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C89" s="7"/>
     </row>
-    <row r="90" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C90" s="7"/>
     </row>
-    <row r="91" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C91" s="7"/>
     </row>
-    <row r="92" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C92" s="7"/>
     </row>
-    <row r="93" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C93" s="7"/>
     </row>
-    <row r="94" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C94" s="7"/>
     </row>
-    <row r="95" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C95" s="7"/>
     </row>
-    <row r="96" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:3" x14ac:dyDescent="0.35">
       <c r="C96" s="7"/>
     </row>
     <row r="97" spans="3:3" x14ac:dyDescent="0.35">

</xml_diff>